<commit_message>
refactor(notebooks): update working directory paths across src and notebook files
</commit_message>
<xml_diff>
--- a/outputs/predictions/Intel Stock Predictions - Real Money.xlsx
+++ b/outputs/predictions/Intel Stock Predictions - Real Money.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21600" windowHeight="10200"/>
+    <workbookView windowWidth="21600" windowHeight="10185"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Date</t>
   </si>
@@ -95,7 +95,7 @@
     <numFmt numFmtId="176" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="177" formatCode="0.0000_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,6 +113,11 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -593,137 +598,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -758,6 +763,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -773,7 +781,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1298,8 +1306,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2"/>
+  <dimension ref="A1:P4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col min="1" max="1" width="18.7142857142857" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.4285714285714" style="2" customWidth="1"/>
@@ -1469,6 +1477,56 @@
         <v>17</v>
       </c>
     </row>
+    <row r="4" spans="1:16">
+      <c r="A4" s="1">
+        <v>46255</v>
+      </c>
+      <c r="B4" s="2">
+        <v>131.81</v>
+      </c>
+      <c r="C4" s="2">
+        <v>135.48</v>
+      </c>
+      <c r="D4" s="2">
+        <v>127.9</v>
+      </c>
+      <c r="E4" s="2">
+        <v>133.99</v>
+      </c>
+      <c r="F4" s="2">
+        <v>124.91</v>
+      </c>
+      <c r="G4" s="2">
+        <v>114.83</v>
+      </c>
+      <c r="H4" s="2">
+        <v>7.58</v>
+      </c>
+      <c r="I4" s="2">
+        <v>133.8772</v>
+      </c>
+      <c r="J4" s="10">
+        <v>133.8856</v>
+      </c>
+      <c r="K4" s="2">
+        <v>133.8687</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0.78</v>
+      </c>
+      <c r="M4" s="4">
+        <v>2.14</v>
+      </c>
+      <c r="N4" s="4">
+        <v>1.67</v>
+      </c>
+      <c r="O4" s="4">
+        <v>3.81</v>
+      </c>
+      <c r="P4" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
chore(data): refresh real-money performance tracking datasheet
</commit_message>
<xml_diff>
--- a/outputs/predictions/Intel Stock Predictions - Real Money.xlsx
+++ b/outputs/predictions/Intel Stock Predictions - Real Money.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>Date</t>
   </si>
@@ -728,7 +728,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -766,6 +766,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1306,8 +1309,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3"/>
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
     <col min="1" max="1" width="18.7142857142857" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.4285714285714" style="2" customWidth="1"/>
@@ -1527,6 +1530,56 @@
         <v>17</v>
       </c>
     </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="1">
+        <v>46256</v>
+      </c>
+      <c r="B5" s="2">
+        <v>131.81</v>
+      </c>
+      <c r="C5" s="2">
+        <v>135.48</v>
+      </c>
+      <c r="D5" s="2">
+        <v>127.9</v>
+      </c>
+      <c r="E5" s="2">
+        <v>133.99</v>
+      </c>
+      <c r="F5" s="2">
+        <v>124.91</v>
+      </c>
+      <c r="G5" s="2">
+        <v>114.83</v>
+      </c>
+      <c r="H5" s="2">
+        <v>7.58</v>
+      </c>
+      <c r="I5" s="2">
+        <v>133.9231</v>
+      </c>
+      <c r="J5" s="8">
+        <v>133.8856</v>
+      </c>
+      <c r="K5" s="2">
+        <v>137.9058</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0.81</v>
+      </c>
+      <c r="M5" s="4">
+        <v>2.14</v>
+      </c>
+      <c r="N5" s="4">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4">
+        <v>0</v>
+      </c>
+      <c r="P5" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>